<commit_message>
demo: tune the 80-row dedup file for deterministic review counts
At the default 0.75 threshold the earlier composition left two duplicate pairs
on the edge (0.754/0.764) and the Lisa/Liza row below it. The fuzzy row is now a
one-letter surname variant (Fernandes vs Fernandez) at ~0.82, and the duplicate
pairs are middle-initial or one first-name spelling apart at 0.83-0.85.

Verified against production clients with the matcher's own score formula at the
default threshold: 9 KAPWA matches (8 exact + 1 fuzzy), 6 duplicate pairs, 59
new clients, and no accidental collisions among the new rows.
</commit_message>
<xml_diff>
--- a/demo/dedup-demo-80.xlsx
+++ b/demo/dedup-demo-80.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="248">
   <si>
     <t>Last Name</t>
   </si>
@@ -148,10 +148,10 @@
     <t>Tricycle driver</t>
   </si>
   <si>
-    <t>Fernandez</t>
-  </si>
-  <si>
-    <t>Lisa</t>
+    <t>Fernandes</t>
+  </si>
+  <si>
+    <t>Liza</t>
   </si>
   <si>
     <t>R</t>
@@ -199,9 +199,6 @@
     <t>S.</t>
   </si>
   <si>
-    <t>1991-08-04</t>
-  </si>
-  <si>
     <t>Quimson</t>
   </si>
   <si>
@@ -217,10 +214,7 @@
     <t>Pinagtulayan</t>
   </si>
   <si>
-    <t>Quimzon</t>
-  </si>
-  <si>
-    <t>Dela Pena</t>
+    <t>Dela P.</t>
   </si>
   <si>
     <t>Valderrama</t>
@@ -235,7 +229,7 @@
     <t>Tigbe</t>
   </si>
   <si>
-    <t>Joceline</t>
+    <t>Jocelyne</t>
   </si>
   <si>
     <t>Malabanan</t>
@@ -1430,7 +1424,7 @@
         <v>61</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E14" t="s">
         <v>60</v>
@@ -1441,19 +1435,19 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" t="s">
         <v>63</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>64</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" t="s">
         <v>66</v>
-      </c>
-      <c r="E15" t="s">
-        <v>67</v>
       </c>
       <c r="F15" t="s">
         <v>30</v>
@@ -1461,19 +1455,19 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" t="s">
         <v>66</v>
-      </c>
-      <c r="E16" t="s">
-        <v>67</v>
       </c>
       <c r="F16" t="s">
         <v>21</v>
@@ -1481,19 +1475,19 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C17" t="s">
         <v>42</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F17" t="s">
         <v>17</v>
@@ -1501,19 +1495,19 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C18" t="s">
         <v>42</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E18" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F18" t="s">
         <v>30</v>
@@ -1521,19 +1515,19 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" t="s">
         <v>75</v>
       </c>
-      <c r="B19" t="s">
+      <c r="D19" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C19" t="s">
+      <c r="E19" t="s">
         <v>77</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="E19" t="s">
-        <v>79</v>
       </c>
       <c r="F19" t="s">
         <v>30</v>
@@ -1541,19 +1535,19 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C20" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>78</v>
-      </c>
       <c r="E20" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F20" t="s">
         <v>41</v>
@@ -1561,39 +1555,39 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" t="s">
         <v>81</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
         <v>83</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="F21" t="s">
         <v>84</v>
-      </c>
-      <c r="E21" t="s">
-        <v>85</v>
-      </c>
-      <c r="F21" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B22" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C22" t="s">
         <v>38</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F22" t="s">
         <v>30</v>
@@ -1601,16 +1595,16 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>85</v>
+      </c>
+      <c r="B23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" t="s">
         <v>87</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="C23" t="s">
-        <v>89</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>90</v>
       </c>
       <c r="E23" t="s">
         <v>55</v>
@@ -1621,16 +1615,16 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B24" t="s">
+        <v>89</v>
+      </c>
+      <c r="C24" t="s">
+        <v>90</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="C24" t="s">
-        <v>92</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="E24" t="s">
         <v>60</v>
@@ -1641,19 +1635,19 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" t="s">
         <v>94</v>
       </c>
-      <c r="B25" t="s">
+      <c r="D25" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C25" t="s">
-        <v>96</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="E25" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F25" t="s">
         <v>30</v>
@@ -1661,16 +1655,16 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" t="s">
         <v>98</v>
       </c>
-      <c r="B26" t="s">
+      <c r="D26" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="C26" t="s">
-        <v>100</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -1681,19 +1675,19 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>100</v>
+      </c>
+      <c r="B27" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" t="s">
+        <v>101</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B27" t="s">
-        <v>64</v>
-      </c>
-      <c r="C27" t="s">
-        <v>103</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="E27" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F27" t="s">
         <v>41</v>
@@ -1701,16 +1695,16 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" t="s">
+        <v>104</v>
+      </c>
+      <c r="C28" t="s">
         <v>105</v>
       </c>
-      <c r="B28" t="s">
+      <c r="D28" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="C28" t="s">
-        <v>107</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="E28" t="s">
         <v>40</v>
@@ -1721,16 +1715,16 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>107</v>
+      </c>
+      <c r="B29" t="s">
+        <v>108</v>
+      </c>
+      <c r="C29" t="s">
         <v>109</v>
       </c>
-      <c r="B29" t="s">
+      <c r="D29" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="C29" t="s">
-        <v>111</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="E29" t="s">
         <v>35</v>
@@ -1741,19 +1735,19 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B30" t="s">
+        <v>111</v>
+      </c>
+      <c r="C30" t="s">
+        <v>112</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C30" t="s">
-        <v>114</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="E30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F30" t="s">
         <v>30</v>
@@ -1761,16 +1755,16 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B31" t="s">
         <v>19</v>
       </c>
       <c r="C31" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E31" t="s">
         <v>16</v>
@@ -1781,19 +1775,19 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" t="s">
+        <v>118</v>
+      </c>
+      <c r="C32" t="s">
         <v>119</v>
       </c>
-      <c r="B32" t="s">
+      <c r="D32" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C32" t="s">
+      <c r="E32" t="s">
         <v>121</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E32" t="s">
-        <v>123</v>
       </c>
       <c r="F32" t="s">
         <v>30</v>
@@ -1801,19 +1795,19 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>122</v>
+      </c>
+      <c r="B33" t="s">
+        <v>123</v>
+      </c>
+      <c r="C33" t="s">
         <v>124</v>
       </c>
-      <c r="B33" t="s">
+      <c r="D33" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C33" t="s">
+      <c r="E33" t="s">
         <v>126</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="E33" t="s">
-        <v>128</v>
       </c>
       <c r="F33" t="s">
         <v>30</v>
@@ -1821,16 +1815,16 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>127</v>
+      </c>
+      <c r="B34" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" t="s">
         <v>129</v>
       </c>
-      <c r="B34" t="s">
+      <c r="D34" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="C34" t="s">
-        <v>131</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="E34" t="s">
         <v>29</v>
@@ -1841,36 +1835,36 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B35" t="s">
+        <v>132</v>
+      </c>
+      <c r="C35" t="s">
+        <v>86</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B35" t="s">
-        <v>134</v>
-      </c>
-      <c r="C35" t="s">
-        <v>88</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="E35" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F35" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>134</v>
+      </c>
+      <c r="B36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C36" t="s">
+        <v>135</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="B36" t="s">
-        <v>91</v>
-      </c>
-      <c r="C36" t="s">
-        <v>137</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>138</v>
       </c>
       <c r="E36" t="s">
         <v>55</v>
@@ -1881,16 +1875,16 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>137</v>
+      </c>
+      <c r="B37" t="s">
+        <v>138</v>
+      </c>
+      <c r="C37" t="s">
         <v>139</v>
       </c>
-      <c r="B37" t="s">
+      <c r="D37" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="C37" t="s">
-        <v>141</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>142</v>
       </c>
       <c r="E37" t="s">
         <v>60</v>
@@ -1901,19 +1895,19 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>141</v>
+      </c>
+      <c r="B38" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" t="s">
+        <v>142</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="B38" t="s">
-        <v>99</v>
-      </c>
-      <c r="C38" t="s">
-        <v>144</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="E38" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F38" t="s">
         <v>30</v>
@@ -1921,16 +1915,16 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>144</v>
+      </c>
+      <c r="B39" t="s">
+        <v>145</v>
+      </c>
+      <c r="C39" t="s">
         <v>146</v>
       </c>
-      <c r="B39" t="s">
+      <c r="D39" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="C39" t="s">
-        <v>148</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="E39" t="s">
         <v>10</v>
@@ -1941,19 +1935,19 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>148</v>
+      </c>
+      <c r="B40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" t="s">
+        <v>149</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B40" t="s">
-        <v>106</v>
-      </c>
-      <c r="C40" t="s">
-        <v>151</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>152</v>
-      </c>
       <c r="E40" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F40" t="s">
         <v>30</v>
@@ -1961,16 +1955,16 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B41" t="s">
+        <v>151</v>
+      </c>
+      <c r="C41" t="s">
+        <v>152</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="C41" t="s">
-        <v>154</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>155</v>
       </c>
       <c r="E41" t="s">
         <v>40</v>
@@ -1981,16 +1975,16 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B42" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C42" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E42" t="s">
         <v>35</v>
@@ -2001,19 +1995,19 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>156</v>
+      </c>
+      <c r="B43" t="s">
+        <v>86</v>
+      </c>
+      <c r="C43" t="s">
+        <v>157</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B43" t="s">
-        <v>88</v>
-      </c>
-      <c r="C43" t="s">
-        <v>159</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>160</v>
-      </c>
       <c r="E43" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F43" t="s">
         <v>30</v>
@@ -2021,16 +2015,16 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>159</v>
+      </c>
+      <c r="B44" t="s">
+        <v>118</v>
+      </c>
+      <c r="C44" t="s">
+        <v>160</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="B44" t="s">
-        <v>120</v>
-      </c>
-      <c r="C44" t="s">
-        <v>162</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>163</v>
       </c>
       <c r="E44" t="s">
         <v>16</v>
@@ -2041,19 +2035,19 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>162</v>
+      </c>
+      <c r="B45" t="s">
+        <v>93</v>
+      </c>
+      <c r="C45" t="s">
+        <v>163</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B45" t="s">
-        <v>95</v>
-      </c>
-      <c r="C45" t="s">
-        <v>165</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="E45" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F45" t="s">
         <v>30</v>
@@ -2061,19 +2055,19 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>165</v>
+      </c>
+      <c r="B46" t="s">
+        <v>128</v>
+      </c>
+      <c r="C46" t="s">
+        <v>166</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B46" t="s">
-        <v>130</v>
-      </c>
-      <c r="C46" t="s">
-        <v>168</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>169</v>
-      </c>
       <c r="E46" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F46" t="s">
         <v>30</v>
@@ -2081,16 +2075,16 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B47" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C47" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E47" t="s">
         <v>29</v>
@@ -2101,19 +2095,19 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>170</v>
+      </c>
+      <c r="B48" t="s">
+        <v>89</v>
+      </c>
+      <c r="C48" t="s">
+        <v>171</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B48" t="s">
-        <v>91</v>
-      </c>
-      <c r="C48" t="s">
-        <v>173</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>174</v>
-      </c>
       <c r="E48" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F48" t="s">
         <v>30</v>
@@ -2121,16 +2115,16 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B49" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C49" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E49" t="s">
         <v>55</v>
@@ -2141,16 +2135,16 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B50" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C50" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E50" t="s">
         <v>60</v>
@@ -2161,19 +2155,19 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B51" t="s">
         <v>19</v>
       </c>
       <c r="C51" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E51" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F51" t="s">
         <v>21</v>
@@ -2181,16 +2175,16 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B52" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C52" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E52" t="s">
         <v>10</v>
@@ -2201,19 +2195,19 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>182</v>
+      </c>
+      <c r="B53" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" t="s">
+        <v>183</v>
+      </c>
+      <c r="D53" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="B53" t="s">
-        <v>125</v>
-      </c>
-      <c r="C53" t="s">
-        <v>185</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>186</v>
-      </c>
       <c r="E53" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F53" t="s">
         <v>30</v>
@@ -2221,16 +2215,16 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>185</v>
+      </c>
+      <c r="B54" t="s">
+        <v>111</v>
+      </c>
+      <c r="C54" t="s">
+        <v>186</v>
+      </c>
+      <c r="D54" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="B54" t="s">
-        <v>113</v>
-      </c>
-      <c r="C54" t="s">
-        <v>188</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>189</v>
       </c>
       <c r="E54" t="s">
         <v>40</v>
@@ -2241,16 +2235,16 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>188</v>
+      </c>
+      <c r="B55" t="s">
+        <v>132</v>
+      </c>
+      <c r="C55" t="s">
+        <v>189</v>
+      </c>
+      <c r="D55" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="B55" t="s">
-        <v>134</v>
-      </c>
-      <c r="C55" t="s">
-        <v>191</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="E55" t="s">
         <v>35</v>
@@ -2261,19 +2255,19 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>191</v>
+      </c>
+      <c r="B56" t="s">
+        <v>118</v>
+      </c>
+      <c r="C56" t="s">
+        <v>192</v>
+      </c>
+      <c r="D56" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B56" t="s">
-        <v>120</v>
-      </c>
-      <c r="C56" t="s">
-        <v>194</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>195</v>
-      </c>
       <c r="E56" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F56" t="s">
         <v>30</v>
@@ -2281,16 +2275,16 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>192</v>
+      </c>
+      <c r="B57" t="s">
+        <v>138</v>
+      </c>
+      <c r="C57" t="s">
+        <v>148</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="B57" t="s">
-        <v>140</v>
-      </c>
-      <c r="C57" t="s">
-        <v>150</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>196</v>
       </c>
       <c r="E57" t="s">
         <v>16</v>
@@ -2301,19 +2295,19 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B58" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C58" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E58" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F58" t="s">
         <v>30</v>
@@ -2321,19 +2315,19 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>196</v>
+      </c>
+      <c r="B59" t="s">
+        <v>145</v>
+      </c>
+      <c r="C59" t="s">
+        <v>197</v>
+      </c>
+      <c r="D59" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="B59" t="s">
-        <v>147</v>
-      </c>
-      <c r="C59" t="s">
-        <v>199</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>200</v>
-      </c>
       <c r="E59" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F59" t="s">
         <v>50</v>
@@ -2341,16 +2335,16 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>199</v>
+      </c>
+      <c r="B60" t="s">
+        <v>89</v>
+      </c>
+      <c r="C60" t="s">
+        <v>200</v>
+      </c>
+      <c r="D60" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="B60" t="s">
-        <v>91</v>
-      </c>
-      <c r="C60" t="s">
-        <v>202</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="E60" t="s">
         <v>29</v>
@@ -2361,19 +2355,19 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>202</v>
+      </c>
+      <c r="B61" t="s">
+        <v>151</v>
+      </c>
+      <c r="C61" t="s">
+        <v>203</v>
+      </c>
+      <c r="D61" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="B61" t="s">
-        <v>153</v>
-      </c>
-      <c r="C61" t="s">
-        <v>205</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>206</v>
-      </c>
       <c r="E61" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F61" t="s">
         <v>30</v>
@@ -2381,16 +2375,16 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>205</v>
+      </c>
+      <c r="B62" t="s">
+        <v>97</v>
+      </c>
+      <c r="C62" t="s">
+        <v>206</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>207</v>
-      </c>
-      <c r="B62" t="s">
-        <v>99</v>
-      </c>
-      <c r="C62" t="s">
-        <v>208</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>209</v>
       </c>
       <c r="E62" t="s">
         <v>55</v>
@@ -2401,39 +2395,39 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B63" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C63" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E63" t="s">
         <v>60</v>
       </c>
       <c r="F63" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B64" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C64" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="E64" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F64" t="s">
         <v>30</v>
@@ -2441,16 +2435,16 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B65" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C65" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E65" t="s">
         <v>10</v>
@@ -2461,19 +2455,19 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>213</v>
+      </c>
+      <c r="B66" t="s">
+        <v>111</v>
+      </c>
+      <c r="C66" t="s">
+        <v>214</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B66" t="s">
-        <v>113</v>
-      </c>
-      <c r="C66" t="s">
-        <v>216</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>217</v>
-      </c>
       <c r="E66" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F66" t="s">
         <v>30</v>
@@ -2481,16 +2475,16 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>216</v>
+      </c>
+      <c r="B67" t="s">
+        <v>63</v>
+      </c>
+      <c r="C67" t="s">
+        <v>217</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="B67" t="s">
-        <v>64</v>
-      </c>
-      <c r="C67" t="s">
-        <v>219</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>220</v>
       </c>
       <c r="E67" t="s">
         <v>40</v>
@@ -2501,16 +2495,16 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B68" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C68" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E68" t="s">
         <v>35</v>
@@ -2521,19 +2515,19 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B69" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C69" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E69" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F69" t="s">
         <v>30</v>
@@ -2541,16 +2535,16 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>223</v>
+      </c>
+      <c r="B70" t="s">
+        <v>128</v>
+      </c>
+      <c r="C70" t="s">
+        <v>224</v>
+      </c>
+      <c r="D70" s="1" t="s">
         <v>225</v>
-      </c>
-      <c r="B70" t="s">
-        <v>130</v>
-      </c>
-      <c r="C70" t="s">
-        <v>226</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>227</v>
       </c>
       <c r="E70" t="s">
         <v>16</v>
@@ -2561,19 +2555,19 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B71" t="s">
         <v>19</v>
       </c>
       <c r="C71" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E71" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F71" t="s">
         <v>30</v>
@@ -2581,19 +2575,19 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B72" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C72" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E72" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F72" t="s">
         <v>30</v>
@@ -2601,16 +2595,16 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B73" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C73" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E73" t="s">
         <v>29</v>
@@ -2621,19 +2615,19 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B74" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C74" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E74" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F74" t="s">
         <v>30</v>
@@ -2641,16 +2635,16 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B75" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C75" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E75" t="s">
         <v>55</v>
@@ -2661,16 +2655,16 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>236</v>
+      </c>
+      <c r="B76" t="s">
+        <v>104</v>
+      </c>
+      <c r="C76" t="s">
+        <v>237</v>
+      </c>
+      <c r="D76" s="1" t="s">
         <v>238</v>
-      </c>
-      <c r="B76" t="s">
-        <v>106</v>
-      </c>
-      <c r="C76" t="s">
-        <v>239</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>240</v>
       </c>
       <c r="E76" t="s">
         <v>60</v>
@@ -2681,19 +2675,19 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>239</v>
+      </c>
+      <c r="B77" t="s">
+        <v>138</v>
+      </c>
+      <c r="C77" t="s">
+        <v>240</v>
+      </c>
+      <c r="D77" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="B77" t="s">
-        <v>140</v>
-      </c>
-      <c r="C77" t="s">
-        <v>242</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>243</v>
-      </c>
       <c r="E77" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F77" t="s">
         <v>30</v>
@@ -2701,16 +2695,16 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B78" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C78" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E78" t="s">
         <v>10</v>
@@ -2721,19 +2715,19 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B79" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C79" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E79" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F79" t="s">
         <v>21</v>
@@ -2741,16 +2735,16 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B80" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C80" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E80" t="s">
         <v>40</v>
@@ -2761,16 +2755,16 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B81" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C81" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E81" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
data(demo): middle names are full or empty, never initials
The deduplication workbooks now carry the same middle-name values as the
production client data: full names where a full name exists, blank otherwise.
The 80-row file's twelve match rows mirror their production records (Castillo
Cruz, Dimagiba Dimayuga, Reyes Poblete; the rest have no middle name), its six
duplicate pairs differ by a full-vs-absent middle, an accent, or a first-name
spelling, and no row carries a single-letter middle. The 15-row fallback file
was corrected the same way.

At the default threshold this keeps 9 KAPWA matches (0.90/0.85, fuzzy 0.80), 6
duplicate pairs (0.85-0.86) and 59 new clients. README and the matching-criteria
document carry the recomputed figures; the demo docs use the new display names.
MSG2
git log --oneline -2
</commit_message>
<xml_diff>
--- a/demo/dedup-demo-80.xlsx
+++ b/demo/dedup-demo-80.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="241">
   <si>
     <t>Last Name</t>
   </si>
@@ -37,7 +37,7 @@
     <t>Nena</t>
   </si>
   <si>
-    <t>C</t>
+    <t>Cruz</t>
   </si>
   <si>
     <t>1975-06-14</t>
@@ -55,7 +55,7 @@
     <t>Carla</t>
   </si>
   <si>
-    <t>D</t>
+    <t>Dimayuga</t>
   </si>
   <si>
     <t>1993-04-19</t>
@@ -73,6 +73,9 @@
     <t>Jose</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>1965-09-18</t>
   </si>
   <si>
@@ -85,9 +88,6 @@
     <t>Rosa</t>
   </si>
   <si>
-    <t>P</t>
-  </si>
-  <si>
     <t>1948-05-02</t>
   </si>
   <si>
@@ -103,18 +103,12 @@
     <t>Partida</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Ramos</t>
   </si>
   <si>
     <t>Pedro</t>
   </si>
   <si>
-    <t>S</t>
-  </si>
-  <si>
     <t>1978-01-09</t>
   </si>
   <si>
@@ -127,9 +121,6 @@
     <t>Maria</t>
   </si>
   <si>
-    <t>L.</t>
-  </si>
-  <si>
     <t>1985-07-22</t>
   </si>
   <si>
@@ -142,6 +133,9 @@
     <t>Reyes</t>
   </si>
   <si>
+    <t>Poblete</t>
+  </si>
+  <si>
     <t>1988-03-21</t>
   </si>
   <si>
@@ -154,9 +148,6 @@
     <t>Liza</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
     <t>1982-02-25</t>
   </si>
   <si>
@@ -181,9 +172,6 @@
     <t>Bangkal</t>
   </si>
   <si>
-    <t>B.</t>
-  </si>
-  <si>
     <t>Buenaventura</t>
   </si>
   <si>
@@ -196,9 +184,6 @@
     <t>Bitungol</t>
   </si>
   <si>
-    <t>S.</t>
-  </si>
-  <si>
     <t>Quimson</t>
   </si>
   <si>
@@ -214,7 +199,7 @@
     <t>Pinagtulayan</t>
   </si>
   <si>
-    <t>Dela P.</t>
+    <t>Dela Pena</t>
   </si>
   <si>
     <t>Valderrama</t>
@@ -238,16 +223,10 @@
     <t>Rolando</t>
   </si>
   <si>
-    <t>Cruz</t>
-  </si>
-  <si>
     <t>1974-09-28</t>
   </si>
   <si>
     <t>San Lorenzo</t>
-  </si>
-  <si>
-    <t>C.</t>
   </si>
   <si>
     <t>Dimaculangan</t>
@@ -1221,27 +1200,27 @@
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
         <v>16</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>25</v>
@@ -1261,7 +1240,7 @@
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>28</v>
@@ -1270,224 +1249,224 @@
         <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
         <v>31</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" t="s">
-        <v>35</v>
-      </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B8" t="s">
+      <c r="E8" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
+      <c r="F8" t="s">
         <v>38</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" t="s">
         <v>42</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B10" t="s">
+      <c r="E10" t="s">
         <v>46</v>
       </c>
-      <c r="C10" t="s">
+      <c r="F10" t="s">
         <v>47</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" t="s">
-        <v>49</v>
-      </c>
-      <c r="F10" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B11" t="s">
+      <c r="E11" t="s">
         <v>52</v>
       </c>
-      <c r="C11" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" t="s">
-        <v>55</v>
-      </c>
       <c r="F11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B12" t="s">
+      <c r="E12" t="s">
         <v>52</v>
       </c>
-      <c r="C12" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" t="s">
-        <v>55</v>
-      </c>
       <c r="F12" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F14" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E15" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F15" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
         <v>62</v>
       </c>
-      <c r="B16" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" t="s">
-        <v>67</v>
-      </c>
       <c r="D16" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E16" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E17" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F17" t="s">
         <v>17</v>
@@ -1495,436 +1474,436 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E18" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F18" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C19" t="s">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E19" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F19" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E20" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F20" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B21" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="E21" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F21" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B22" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C22" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="E22" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B23" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C23" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F23" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B24" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C24" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E24" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F24" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="B25" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C25" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E25" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F25" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="B26" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C26" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B27" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C27" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="E27" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F27" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="B28" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C28" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="E28" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F28" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="B29" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C29" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="E29" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F29" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="B30" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="E30" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F30" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B31" t="s">
         <v>19</v>
       </c>
       <c r="C31" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="E31" t="s">
         <v>16</v>
       </c>
       <c r="F31" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B32" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C32" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="E32" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="F32" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B33" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C33" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="E33" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="F33" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B34" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C34" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="E34" t="s">
         <v>29</v>
       </c>
       <c r="F34" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B35" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C35" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="E35" t="s">
+        <v>71</v>
+      </c>
+      <c r="F35" t="s">
         <v>77</v>
-      </c>
-      <c r="F35" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B36" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C36" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="E36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F36" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B37" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C37" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="E37" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F37" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B38" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="E38" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F38" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B39" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C39" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="E39" t="s">
         <v>10</v>
@@ -1935,156 +1914,156 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B40" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C40" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="E40" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F40" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="B41" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C41" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="E41" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F41" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B42" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C42" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="E42" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F42" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="B43" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C43" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="E43" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F43" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="B44" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C44" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="E44" t="s">
         <v>16</v>
       </c>
       <c r="F44" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C45" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="E45" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="F45" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="B46" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C46" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="E46" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="F46" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="B47" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C47" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="E47" t="s">
         <v>29</v>
@@ -2095,399 +2074,399 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B48" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C48" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="E48" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F48" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="B49" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C49" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="E49" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F49" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B50" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C50" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="E50" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F50" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="B51" t="s">
         <v>19</v>
       </c>
       <c r="C51" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="E51" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F51" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="B52" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C52" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="E52" t="s">
         <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="B53" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C53" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="E53" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F53" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="B54" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C54" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="E54" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F54" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B55" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C55" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="E55" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F55" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="B56" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C56" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="E56" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F56" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="B57" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C57" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="E57" t="s">
         <v>16</v>
       </c>
       <c r="F57" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="B58" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C58" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="E58" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="F58" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="B59" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C59" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="E59" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="F59" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="B60" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C60" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="E60" t="s">
         <v>29</v>
       </c>
       <c r="F60" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B61" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C61" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="E61" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F61" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B62" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C62" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="E62" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F62" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="B63" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C63" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="E63" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F63" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="B64" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C64" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="E64" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F64" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="B65" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C65" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="E65" t="s">
         <v>10</v>
       </c>
       <c r="F65" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B66" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C66" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="E66" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F66" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="B67" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C67" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="E67" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F67" t="s">
         <v>17</v>
@@ -2495,159 +2474,159 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B68" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C68" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="E68" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F68" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B69" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C69" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E69" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F69" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="B70" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C70" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="E70" t="s">
         <v>16</v>
       </c>
       <c r="F70" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="B71" t="s">
         <v>19</v>
       </c>
       <c r="C71" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="E71" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="F71" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B72" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C72" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="E72" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="F72" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B73" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C73" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="E73" t="s">
         <v>29</v>
       </c>
       <c r="F73" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="B74" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C74" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="E74" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="F74" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B75" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C75" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="E75" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F75" t="s">
         <v>11</v>
@@ -2655,122 +2634,122 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="B76" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C76" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="E76" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F76" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="B77" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C77" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="E77" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F77" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="B78" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C78" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="E78" t="s">
         <v>10</v>
       </c>
       <c r="F78" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="B79" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C79" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="E79" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F79" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B80" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C80" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="E80" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F80" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="B81" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C81" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="E81" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F81" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>